<commit_message>
fix: Director view - convert docente_id to user_id for PlanificacionPersonal + dialog for multi-docente selection
</commit_message>
<xml_diff>
--- a/dist/spa/templates/plantilla_preguntas.xlsx
+++ b/dist/spa/templates/plantilla_preguntas.xlsx
@@ -397,15 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="8.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
@@ -445,39 +445,103 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>Cuál es la capital constitucional de Bolivia?</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>SELECCION_UNICA</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Sucre</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>La Paz</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>Santa Cruz</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Cochabamba</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
+        <v>FACIL</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Cuáles son los servicios fundamentales del sistema de salud? (Seleccione todas las correctas)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SELECCION_MULTIPLE</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Atención primaria</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Prevención</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Rehabilitación</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Solo consulta externa</v>
+      </c>
+      <c r="G3" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="H3" t="str">
+        <v>MEDIO</v>
+      </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
+      <c r="J3" t="str">
+        <v>A;B;C</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>El corazón humano tiene cuatro cavidades.</v>
+      </c>
+      <c r="B4" t="str">
+        <v>FALSO_VERDADERO</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verdadero</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Falso</v>
+      </c>
+      <c r="E4" t="str">
         <v/>
       </c>
-      <c r="J2" t="str">
+      <c r="F4" t="str">
         <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>FACIL</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>